<commit_message>
Update LSP management spreadsheet
</commit_message>
<xml_diff>
--- a/data/20251229_LSP管理.xlsx
+++ b/data/20251229_LSP管理.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hiraizumitatsuya/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3278" documentId="13_ncr:1_{118E22AB-A700-4546-AC50-A03A5FE8C08A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34C2A018-3B5E-44AD-9CB6-B4B21DF9FC8A}"/>
+  <xr:revisionPtr revIDLastSave="3303" documentId="13_ncr:1_{118E22AB-A700-4546-AC50-A03A5FE8C08A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9BA3037-CA79-4151-95BE-E62830B49956}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3303" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3321" uniqueCount="419">
   <si>
     <t>日付</t>
   </si>
@@ -1274,6 +1274,15 @@
   </si>
   <si>
     <t>JAL106</t>
+  </si>
+  <si>
+    <t>JAL23７</t>
+  </si>
+  <si>
+    <t>JAL639</t>
+  </si>
+  <si>
+    <t>JAL631</t>
   </si>
   <si>
     <t>総額</t>
@@ -61931,19 +61940,19 @@
         <v>306</v>
       </c>
       <c r="D239" s="12" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="E239" s="12" t="s">
         <v>307</v>
       </c>
       <c r="F239" s="13">
-        <v>0.43055555555555558</v>
+        <v>0.60763888888888884</v>
       </c>
       <c r="G239" s="12" t="s">
         <v>359</v>
       </c>
       <c r="H239" s="13">
-        <v>0.4861111111111111</v>
+        <v>0.65972222222222221</v>
       </c>
       <c r="I239" s="26"/>
       <c r="J239" s="15" t="s">
@@ -61952,9 +61961,7 @@
       <c r="K239" s="22">
         <v>0</v>
       </c>
-      <c r="L239" s="15" t="s">
-        <v>310</v>
-      </c>
+      <c r="L239" s="15"/>
       <c r="M239" s="15"/>
     </row>
     <row r="240" spans="1:13">
@@ -61962,7 +61969,7 @@
         <v>255</v>
       </c>
       <c r="B240" s="42">
-        <v>46286</v>
+        <v>46321</v>
       </c>
       <c r="C240" s="12" t="s">
         <v>306</v>
@@ -61974,13 +61981,13 @@
         <v>359</v>
       </c>
       <c r="F240" s="13">
-        <v>0.72916666666666663</v>
+        <v>0.71875</v>
       </c>
       <c r="G240" s="12" t="s">
         <v>307</v>
       </c>
       <c r="H240" s="13">
-        <v>0.78125</v>
+        <v>0.77083333333333337</v>
       </c>
       <c r="I240" s="26"/>
       <c r="J240" s="15" t="s">
@@ -61989,76 +61996,146 @@
       <c r="K240" s="22">
         <v>0</v>
       </c>
-      <c r="L240" s="15" t="s">
-        <v>310</v>
-      </c>
+      <c r="L240" s="15"/>
       <c r="M240" s="15"/>
     </row>
-    <row r="241" spans="1:13" ht="14.25">
+    <row r="241" spans="1:13">
       <c r="A241" s="14">
         <v>256</v>
       </c>
-      <c r="B241" s="42"/>
-      <c r="C241" s="61"/>
-      <c r="D241" s="61"/>
-      <c r="E241" s="61"/>
-      <c r="F241" s="62"/>
-      <c r="G241" s="61"/>
-      <c r="H241" s="62"/>
-      <c r="I241" s="61"/>
-      <c r="J241" s="15"/>
-      <c r="K241" s="22"/>
+      <c r="B241" s="42">
+        <v>46432</v>
+      </c>
+      <c r="C241" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="D241" s="12" t="s">
+        <v>409</v>
+      </c>
+      <c r="E241" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="F241" s="13">
+        <v>0.78819444444444442</v>
+      </c>
+      <c r="G241" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="H241" s="13">
+        <v>0.86805555555555558</v>
+      </c>
+      <c r="I241" s="26"/>
+      <c r="J241" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="K241" s="22">
+        <v>0</v>
+      </c>
       <c r="L241" s="15"/>
       <c r="M241" s="15"/>
     </row>
-    <row r="242" spans="1:13" ht="14.25">
+    <row r="242" spans="1:13">
       <c r="A242" s="14">
         <v>257</v>
       </c>
-      <c r="B242" s="42"/>
-      <c r="C242" s="61"/>
-      <c r="D242" s="61"/>
-      <c r="E242" s="61"/>
-      <c r="F242" s="62"/>
-      <c r="G242" s="61"/>
-      <c r="H242" s="62"/>
-      <c r="I242" s="61"/>
-      <c r="J242" s="15"/>
-      <c r="K242" s="22"/>
+      <c r="B242" s="42">
+        <v>46433</v>
+      </c>
+      <c r="C242" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="D242" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="E242" s="12" t="s">
+        <v>359</v>
+      </c>
+      <c r="F242" s="13">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="G242" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="H242" s="13">
+        <v>0.64236111111111116</v>
+      </c>
+      <c r="I242" s="26"/>
+      <c r="J242" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="K242" s="22">
+        <v>0</v>
+      </c>
       <c r="L242" s="15"/>
       <c r="M242" s="15"/>
     </row>
-    <row r="243" spans="1:13" ht="14.25">
+    <row r="243" spans="1:13">
       <c r="A243" s="14">
         <v>258</v>
       </c>
-      <c r="B243" s="42"/>
-      <c r="C243" s="61"/>
-      <c r="D243" s="61"/>
-      <c r="E243" s="61"/>
-      <c r="F243" s="62"/>
-      <c r="G243" s="61"/>
-      <c r="H243" s="62"/>
-      <c r="I243" s="61"/>
-      <c r="J243" s="15"/>
-      <c r="K243" s="22"/>
+      <c r="B243" s="42">
+        <v>46446</v>
+      </c>
+      <c r="C243" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="D243" s="12" t="s">
+        <v>410</v>
+      </c>
+      <c r="E243" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="F243" s="13">
+        <v>0.53819444444444442</v>
+      </c>
+      <c r="G243" s="12" t="s">
+        <v>388</v>
+      </c>
+      <c r="H243" s="13">
+        <v>0.61111111111111116</v>
+      </c>
+      <c r="I243" s="26"/>
+      <c r="J243" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="K243" s="22">
+        <v>0</v>
+      </c>
       <c r="L243" s="15"/>
       <c r="M243" s="15"/>
     </row>
-    <row r="244" spans="1:13" ht="14.25">
+    <row r="244" spans="1:13">
       <c r="A244" s="14">
         <v>259</v>
       </c>
-      <c r="B244" s="42"/>
-      <c r="C244" s="61"/>
-      <c r="D244" s="61"/>
-      <c r="E244" s="61"/>
-      <c r="F244" s="62"/>
-      <c r="G244" s="61"/>
-      <c r="H244" s="62"/>
-      <c r="I244" s="61"/>
-      <c r="J244" s="15"/>
-      <c r="K244" s="22"/>
+      <c r="B244" s="42">
+        <v>46447</v>
+      </c>
+      <c r="C244" s="12" t="s">
+        <v>306</v>
+      </c>
+      <c r="D244" s="12" t="s">
+        <v>396</v>
+      </c>
+      <c r="E244" s="12" t="s">
+        <v>359</v>
+      </c>
+      <c r="F244" s="13">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="G244" s="12" t="s">
+        <v>307</v>
+      </c>
+      <c r="H244" s="13">
+        <v>0.64236111111111116</v>
+      </c>
+      <c r="I244" s="26"/>
+      <c r="J244" s="15" t="s">
+        <v>371</v>
+      </c>
+      <c r="K244" s="22">
+        <v>0</v>
+      </c>
       <c r="L244" s="15"/>
       <c r="M244" s="15"/>
     </row>
@@ -62387,7 +62464,7 @@
     </row>
     <row r="274" spans="10:11">
       <c r="J274" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="K274" s="11">
         <f>SUM(テーブル4[料金])</f>
@@ -62396,11 +62473,11 @@
     </row>
     <row r="275" spans="10:11">
       <c r="J275" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="K275">
         <f>COUNTA(テーブル4[料金])*5</f>
-        <v>1175</v>
+        <v>1195</v>
       </c>
     </row>
     <row r="276" spans="10:11">
@@ -62409,16 +62486,16 @@
       </c>
       <c r="K276">
         <f>COUNTA(テーブル4[料金])</f>
-        <v>235</v>
+        <v>239</v>
       </c>
     </row>
     <row r="277" spans="10:11">
       <c r="J277" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="K277" s="41">
         <f>K274/K275</f>
-        <v>1160.4459574468085</v>
+        <v>1141.0242677824267</v>
       </c>
     </row>
     <row r="289" spans="1:8">
@@ -62496,7 +62573,7 @@
         <v>0.43402777777777779</v>
       </c>
       <c r="H291" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="292" spans="1:8">
@@ -62548,7 +62625,7 @@
         <v>0.57291666666666663</v>
       </c>
       <c r="H293" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
     </row>
     <row r="294" spans="1:8">
@@ -62652,7 +62729,7 @@
         <v>0.91666666666666663</v>
       </c>
       <c r="H297" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
     </row>
     <row r="300" spans="1:8">
@@ -62886,7 +62963,7 @@
         <v>0.375</v>
       </c>
       <c r="H309" s="51" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="I309" s="52"/>
     </row>
@@ -62940,7 +63017,7 @@
         <v>0.54513888888888884</v>
       </c>
       <c r="H311" s="49" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="I311" s="52"/>
     </row>
@@ -63075,7 +63152,7 @@
         <v>0.78472222222222221</v>
       </c>
       <c r="H316" s="54" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="I316" s="56"/>
     </row>

</xml_diff>